<commit_message>
audit(ledger): close F76 live — focus ring verified on production deploy d364718
Merged qa/fixes-20260810 to main and deployed at Dexter's explicit instruction.
Live https://imjustdex.com/ and /brand/ serve home-augment.css?v=phase32; on the
live homepage .sm-submit matches :focus-visible and computes 'solid 2px
rgb(204, 0, 0)' at -2px offset over the --ink face.

F76: ISSUE/High -> PASS (closed live). 77 PASS / 1 ISSUE / 1 N/A / 3 partial.
Only F82 (Low, doc-vs-CSS parity) remains open, still NEEDS DEXTER.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,11 +48,6 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="001A1A1A"/>
       <sz val="10"/>
     </font>
@@ -73,7 +68,7 @@
       <color rgb="00C0211B"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -93,11 +88,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6E7C9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E0625B"/>
       </patternFill>
     </fill>
     <fill>
@@ -147,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -168,20 +158,16 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4555,12 +4541,12 @@
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>ISSUE — .subscribe-manifesto .sm-submit (homepage + /brand/ subscribe submit) has base and :hover styling but NO :focus-visible rule, so the site's primary conversion control shows no focus indicator for keyboard users (WCAG 2.4.7 AA). Every sibling control is covered — .sm-input directly above it has the rule, and .sm-submit is even named in home-augment.css's prefers-reduced-motion block — so this is an omission, not a decision. Missed by prior runs because F76 was tested at sheet level (':focus-visible present in all 8 stylesheets') rather than per control; enumerating all 34 interactive elements on the homepage against the 27 focus selectors in the live CSS surfaced it.</t>
-        </is>
-      </c>
-      <c r="I79" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>PASS (closed live 2026-08-10) — was ISSUE/High: .subscribe-manifesto .sm-submit (homepage + /brand/ subscribe submit) had base and :hover styling but NO :focus-visible rule, so the site's primary conversion control showed no focus indicator for keyboard users (WCAG 2.4.7 AA). Every sibling control was covered — .sm-input directly above it had the rule, and .sm-submit was even named in home-augment.css's prefers-reduced-motion block — so it was an omission, not a decision. Missed by prior runs because F76 was tested at sheet level (':focus-visible present in all 8 stylesheets') rather than per control. Fixed and deployed same day; see p3/p4.</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>High (resolved)</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
@@ -4570,7 +4556,7 @@
       </c>
       <c r="K79" s="6" t="inlineStr">
         <is>
-          <t>PASS (runtime-verified on build, 2026-08-10 12:5x) — keyboard Tab from .sm-input lands on .sm-submit; el.matches(':focus-visible') === true and the computed outline is 'solid 2px rgb(204, 0, 0)' at outline-offset -2px, served from home-augment.css?v=phase32 on the local dev build. Ring contrast against the button's --ink face passes SC 1.4.11 in both modes (5.17:1 dark, 3.44:1 light). This supersedes the morning run's build-only verification, which could not exercise focus modality (0x0 viewport). Live-verify on the next scrub after merge — live CSS still ships phase25 without the rule.</t>
+          <t>PASS (live-verified 2026-08-10 13:31 CDT, deploy d364718) — merged to main and shipped at Dexter's explicit instruction. Live https://imjustdex.com/ and /brand/ both reference home-augment.css?v=phase32; the live sheet serves the rule; on the live homepage .sm-submit matches ':focus-visible' and computes outline 'solid 2px rgb(204, 0, 0)' at outline-offset -2px over the button's --ink face (rgb(5,5,5)). Ring contrast passes SC 1.4.11 in both modes (5.17:1 dark, 3.44:1 light). Verification ladder this day: build-verified 05:06 → runtime-verified on dev build 13:05 → live-verified on production 13:31.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4862,7 @@
           <t>ISSUE — DESIGN-SYSTEM.md:115 lists "Reading progress bar (`var(--accent)`)" as a permitted accent use, but css/article.css:882 ships `.reading-progress { background: var(--ink) }`. Commit 68b0c1d (2026-04-10) recolored it on purpose and left the reason in the CSS: "Reading progress uses --ink rather than --accent so the red accent stays reserved for section heads, callouts, and underlines. A red bar at the top of the viewport was competing with the masthead." That commit rewrote 136 lines of DESIGN-SYSTEM.md but missed this bullet, which dates to c75ded9 earlier the same day. The CSS is correct; the doc line is stale. Live-confirmed today: bar computes rgb(5,5,5) = --ink.</t>
         </is>
       </c>
-      <c r="I85" s="8" t="inlineStr">
+      <c r="I85" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -4908,7 +4894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4916,14 +4902,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Phase 2 Test Results</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>— P2 (test) —</t>
         </is>
@@ -4935,8 +4921,8 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="B4" s="11" t="n">
-        <v>76</v>
+      <c r="B4" s="10" t="n">
+        <v>77</v>
       </c>
     </row>
     <row r="5">
@@ -4945,8 +4931,8 @@
           <t>ISSUE</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>2</v>
+      <c r="B5" s="11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -4955,7 +4941,7 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4965,12 +4951,12 @@
           <t>PENDING</t>
         </is>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B7" s="13" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>— P4 (re-test) —</t>
         </is>
@@ -4982,7 +4968,7 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="10" t="n">
         <v>78</v>
       </c>
     </row>
@@ -4992,12 +4978,12 @@
           <t>PENDING</t>
         </is>
       </c>
-      <c r="B11" s="14" t="n">
+      <c r="B11" s="13" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>— Issues by severity (found) —</t>
         </is>
@@ -5006,45 +4992,35 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="n">
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="B15" s="16" t="n">
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Resolved (P4 PASS)</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Resolved (P4 PASS)</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="n">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Still open</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>Still open</t>
-        </is>
-      </c>
-      <c r="B18" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Total features: 82</t>
         </is>

</xml_diff>

<commit_message>
content(nav): clear the 4 stale ghost flags in prev/next frontmatter [F41/F81]
next-verse.prev, not-the-same-as-alive.next, pulpit.next, and
should-have-killed-it.next all still carried ghost: true pointing at essays
that have since published — the flags asserted a coming-soon state that
stopped being true months ago.

They were already inert: ArticleLayout derives the effective ghost state from
the target's real live status, so all four rendered as normal rel=next links.
Rendered output is byte-identical before and after this change, verified
against the build. This fixes the data to say what the render already did.

Flipped to false rather than deleted, matching the ghost: false convention the
other 13 prev/next blocks carry. Frontmatter only — one line per file, no prose
touched. Collection-wide: zero ghost: true remain, zero ghost teasers render
across all 16, 15 rel=next head links.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -2668,7 +2668,7 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>Authored prev/next render correctly on all 16. Ghost/teaser path PENDING — requires a future-dated entry; none exists. 2026-08-10 PM: the derive-from-live-status fix (p3) live-verified — 4 essays still carry stale ghost:true frontmatter (next-verse.prev→job, not-the-same-as-alive.next→music-that-raised-me, pulpit.next→the-stone, should-have-killed-it.next→job) and all 4 render as real .article-nav-link anchors with rel=prev/next plus matching &lt;link rel&gt; head tags. No ghost teaser leaks.</t>
+          <t>Authored prev/next render correctly on all 16. Ghost/teaser path PENDING — requires a future-dated entry; none exists. 2026-08-10 PM: the derive-from-live-status fix (p3) live-verified, then the underlying data cleaned — the 4 stale ghost:true flags are gone (see F81). Zero `ghost: true` remain in the collection; all 16 essays render real .article-nav-link anchors, 15 rel=next head links (newest correctly has none), zero article-nav-ghost teasers.</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr"/>
@@ -4786,12 +4786,12 @@
       <c r="I84" s="6" t="inlineStr"/>
       <c r="J84" s="4" t="inlineStr">
         <is>
-          <t>FIX (2026-08-07, Dexter's call — resolution 1 of 3): added next{slug:'send-someone-else', title:'Send Someone Else', ghost:false} to show-me-your-glory.mdx. Editorial decision made by Dexter, not by the loop. NOTE this intentionally creates the corpus's first NON-RECIPROCAL pair: glory now points forward to send-someone-else, but send-someone-else.prev still points back to 'some' — the deliberate pulpit → some → send-someone-else calling thread. That asymmetry is by design; do not 'fix' it in a future run.</t>
+          <t>FIX (2026-08-10, Dexter's call): flipped the 4 stale `ghost: true` frontmatter flags to false — next-verse.prev→job, not-the-same-as-alive.next→music-that-raised-me, pulpit.next→the-stone, should-have-killed-it.next→job. All 4 targets had gone live, leaving the flags asserting a coming-soon state that was no longer true. Flipped rather than deleted, to match the `ghost: false` convention the other 13 prev/next blocks already carry. Frontmatter only — one line per file, zero prose touched.</t>
         </is>
       </c>
       <c r="K84" s="6" t="inlineStr">
         <is>
-          <t>PASS (verified against build, then live) — show-me-your-glory emits &lt;link rel=next&gt; to send-someone-else and renders a normal 'Next Essay → Send Someone Else' nav (no ghost class, since ArticleLayout derives ghost from the target's real live status). Forward chain now walks all 16 published essays end to end: reckonings → … → show-me-your-glory → send-someone-else. Zero non-newest essays lack a next.</t>
+          <t>PASS (verified against build, then live) — rendered nav is byte-identical before and after the flip, confirming the flags were already inert under ArticleLayout's derive-from-live-status logic: same .article-nav-prev/.article-nav-next anchors, same &lt;link rel=next&gt; targets on all 4 essays. Collection-wide: zero `ghost: true` remain, zero .article-nav-ghost teasers render across all 16, 15 rel=next head links. The data now says what the render already did.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
audit(ledger): 2026-08-13 scrub — 82->84 rows, F77 fixed, F83/F84 opened BLOCKED
Full regression: 27 rows re-verified live with dated evidence. One HIGH
found and fixed (F77, dark-mode Latest chip 3.44:1 -> 5.17:1). Two rows
opened BLOCKED for Dexter's design call: F83 (four dark-mode hover rules
on the same accent fill) and F84 (the chip vs the doc's Prohibited
accent list, the half F82 did not audit).
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$3:$K$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$3:$K$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -63,7 +63,7 @@
       <color rgb="00C0211B"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +88,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2E2DE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4B9B5"/>
       </patternFill>
     </fill>
   </fills>
@@ -117,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -142,6 +147,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -507,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K85"/>
+  <dimension ref="A1:K87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -734,7 +740,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>PASS — toggle cycles dark→light→dark; dxmode cookie written both ways; label + aria-pressed + bg/ink all update. Reconfirmed 2026-08-10 PM across 3 consecutive clicks.</t>
+          <t>PASS — toggle cycles dark→light→dark; dxmode cookie written both ways; label + aria-pressed + bg/ink all update. Reconfirmed 2026-08-10 PM across 3 consecutive clicks. | 2026-08-13 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways; --bg/--ink/--accent-text all re-resolved (#060606/#f3f0e8/#ff4d4d dark, #f4f4f1/#050505/#c00 light).</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr"/>
@@ -783,7 +789,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: skip link is first focusable; activating it lands document.activeElement on MAIN#archive (home) / MAIN#article (essay); tabindex=-1 present on both landmarks. The 2c7d88d fix holds in production.</t>
+          <t>PASS — live-verified 2026-08-10: skip link is first focusable; activating it lands document.activeElement on MAIN#archive (home) / MAIN#article (essay); tabindex=-1 present on both landmarks. The 2c7d88d fix holds in production. | 2026-08-13 re-verified live: tab-target verified on live: .skip-link reveals from left:-999px to a 83x69 box at (12,12), cream-on-ink 17.79:1; activating it moved document.activeElement to MAIN#archive (tabindex=-1). Article pages target #article.</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
@@ -987,7 +993,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>PASS — /img/favicon-32.png + /img/apple-touch-icon.png 200 on every referenced path</t>
+          <t>PASS — /img/favicon-32.png + /img/apple-touch-icon.png 200 on every referenced path | 2026-08-13 re-verified live: /img/favicon-32.png and /img/apple-touch-icon.png both 200, immutable-cached.</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr"/>
@@ -1036,7 +1042,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>PASS — Anton + IBM Plex Sans self-hosted, preloaded, document.fonts status 'loaded'; CSP font-src intact</t>
+          <t>PASS — Anton + IBM Plex Sans self-hosted, preloaded, document.fonts status 'loaded'; CSP font-src intact | 2026-08-13 re-verified live: document.fonts.status 'loaded'; Anton 400, IBM Plex Sans 400 + 700 all report 'loaded' on home and article. No FOUT observed.</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr"/>
@@ -1138,7 +1144,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>PASS — title/description/canonical on all 21 routes; every canonical on imjustdex.com</t>
+          <t>PASS — title/description/canonical on all 21 routes; every canonical on imjustdex.com | 2026-08-13 re-verified live: title/description/canonical present and pointing at imjustdex.com on all 16 articles + home/about/brand/phase0.</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr"/>
@@ -1187,7 +1193,7 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>PASS — og+twitter complete on all 21; all 19 OG images 200 (16 essays + home/about/phase0/brand)</t>
+          <t>PASS — og+twitter complete on all 21; all 19 OG images 200 (16 essays + home/about/phase0/brand) | 2026-08-13 re-verified live: og:title/og:description/og:image/twitter:card present on all 16 articles; og:image matches the JSON-LD image URL exactly (same cache-bust) on every one.</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr"/>
@@ -1240,7 +1246,7 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>PASS — WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor)</t>
+          <t>PASS — WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor) | 2026-08-13 re-verified live: homepage @graph carries WebSite + Person; Person has all of name/url/sameAs/jobTitle/worksFor.</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr"/>
@@ -1289,7 +1295,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>PASS — ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description)</t>
+          <t>PASS — ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description) | 2026-08-13 re-verified live: /about/ ProfilePage mainEntity is @type Person with name/url/jobTitle/worksFor/sameAs/description — zero missing fields.</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
@@ -1338,7 +1344,7 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>PASS — BlogPosting complete on all 16 (headline, description, datePublished, dateModified, author Person, publisher Organization+logo, mainEntityOfPage, image, url, inLanguage, wordCount); image == og:image exactly, no og-default drift</t>
+          <t>PASS — BlogPosting complete on all 16 (headline, description, datePublished, dateModified, author Person, publisher Organization+logo, mainEntityOfPage, image, url, inLanguage, wordCount); image == og:image exactly, no og-default drift | 2026-08-13 re-verified live: all 16 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount); zero og-default.png drift.</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr"/>
@@ -1436,7 +1442,7 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>PASS — robots.txt Allow / + Sitemap → sitemap-index.xml</t>
+          <t>PASS — robots.txt Allow / + Sitemap → sitemap-index.xml | 2026-08-13 re-verified live: /robots.txt 200, Sitemap directive -&gt; https://imjustdex.com/sitemap-index.xml.</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr"/>
@@ -1485,7 +1491,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>PASS — sitemap-0.xml 20 locs = exactly the published set + about/brand/phase0; no missing, no orphans</t>
+          <t>PASS — sitemap-0.xml 20 locs = exactly the published set + about/brand/phase0; no missing, no orphans | 2026-08-13 re-verified live: /sitemap-index.xml -&gt; sitemap-0.xml; sitemap-0 lists 20 URLs covering all 16 articles + /, /about/, /brand/, /phase0/. Zero missing.</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr"/>
@@ -1587,7 +1593,7 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>PASS — Entry No. 16 / Week of July 5, 2026, LatestBar → newest essay</t>
+          <t>PASS — Entry No. 16 / Week of July 5, 2026, LatestBar → newest essay | 2026-08-13 re-verified live: LatestBar reads 'Entry No. 16 / Week of July 5, 2026' and links to /words/send-someone-else/ (the newest). NOTE: its .latest-tag chip is the F77 finding this run.</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr"/>
@@ -1689,7 +1695,7 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>PASS — Faith 13 / Identity 09 / Art 03, verified against frontmatter lanes; 16 articles</t>
+          <t>PASS — Faith 13 / Identity 09 / Art 03, verified against frontmatter lanes; 16 articles | 2026-08-13 re-verified live: lane-index counts Faith 13 / Identity 09 / Art 03 — non-negative, zero-padded, and consistent with 16 essays counted per lane (15 .plate-lane chips + 1 .lead-badge-lane).</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
@@ -2358,7 +2364,7 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>PASS — bar width 0→249→698→1153px and aria-valuenow 0→30→69→100 across the scroll range. 2026-08-10 PM re-check: structural half re-verified (progress.js math recomputed by hand at 50% scroll = 51.5%; .article-body + .reading-progress present; role/aria-label/aria-valuemin/max initialized on load). Runtime paint not re-exercisable this run — the browser pane reports document.visibilityState 'hidden', so requestAnimationFrame never fires and the CSS width transition stays frozen at 0. Harness limitation, not a site regression.</t>
+          <t>PASS — bar width 0→249→698→1153px and aria-valuenow 0→30→69→100 across the scroll range. 2026-08-10 PM re-check: structural half re-verified (progress.js math recomputed by hand at 50% scroll = 51.5%; .article-body + .reading-progress present; role/aria-label/aria-valuemin/max initialized on load). Runtime paint not re-exercisable this run — the browser pane reports document.visibilityState 'hidden', so requestAnimationFrame never fires and the CSS width transition stays frozen at 0. Harness limitation, not a site regression. | 2026-08-13 re-verified live: reading-progress present on articles at 3px, background var(--ink) rgb(5,5,5) — correct per F82; the doc bullet claiming --accent was struck 2026-08-10.</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr"/>
@@ -3137,7 +3143,7 @@
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>PASS — Atom 16 entries = 16 published; namespace + entries valid</t>
+          <t>PASS — Atom 16 entries = 16 published; namespace + entries valid | 2026-08-13 re-verified live: /feed.xml 200, Atom namespace, 16 &lt;entry&gt; elements — exactly matching the 16 articles on the homepage, zero set difference either direction.</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr"/>
@@ -3190,7 +3196,7 @@
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>PASS — feed.xsl 200 and &lt;?xml-stylesheet?&gt; PI present</t>
+          <t>PASS — feed.xsl 200 and &lt;?xml-stylesheet?&gt; PI present | 2026-08-13 re-verified live: /feed.xsl 200 and referenced via &lt;?xml-stylesheet?&gt; in the feed prolog.</t>
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr"/>
@@ -3667,7 +3673,7 @@
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>PASS — healthscrub+20260807@imjustdex.com → 200 subscribed in 1.53s</t>
+          <t>PASS — healthscrub+20260807@imjustdex.com → 200 subscribed in 1.53s | 2026-08-13 re-verified live: live smoke test POST /api/subscribe returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.16s using healthscrub+20260813@imjustdex.com.</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr"/>
@@ -3879,7 +3885,7 @@
       </c>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>PASS — /about, /phase0 and all 16 /words/&lt;slug&gt; → single 301 to trailing-slash canonical</t>
+          <t>PASS — /about, /phase0 and all 16 /words/&lt;slug&gt; → single 301 to trailing-slash canonical | 2026-08-13 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200; /sitemap.xml correctly 404 post-cutover.</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr"/>
@@ -4038,7 +4044,7 @@
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>PASS — /api/subscribe rewrite reaches the function (405 on GET, 400/200 on POST)</t>
+          <t>PASS — /api/subscribe rewrite reaches the function (405 on GET, 400/200 on POST) | 2026-08-13 re-verified live: /api/subscribe rewrite reached the Netlify function and returned a Mailchimp success body.</t>
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr"/>
@@ -4091,7 +4097,7 @@
       </c>
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>PASS — unmatched route → 404 with the branded body</t>
+          <t>PASS — unmatched route → 404 with the branded body | 2026-08-13 re-verified live: /404 returns 200 with the bespoke 'Nothing to Document Here' body and noindex; /DESIGN-SYSTEM.md and /audit/features.json both 404 (docs not leaking).</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr"/>
@@ -4144,7 +4150,7 @@
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>PASS — CSP present and strict on every page; per-route /brand/ + /feed.xml overrides intact; 0 inline &lt;style&gt; in built Astro HTML</t>
+          <t>PASS — CSP present and strict on every page; per-route /brand/ + /feed.xml overrides intact; 0 inline &lt;style&gt; in built Astro HTML | 2026-08-13 re-verified live: CSP header present and ENFORCING — a runtime &lt;style&gt; injection was blocked by style-src 'self' during F77 verification, which is direct proof the policy is live, not just declared. Per-route /brand/ and /feed.xml relaxations by design.</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr"/>
@@ -4197,7 +4203,7 @@
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>PASS — X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy, Permissions-Policy, COOP, CORP on all 21 routes</t>
+          <t>PASS — X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy, Permissions-Policy, COOP, CORP on all 21 routes | 2026-08-13 re-verified live: all 5 security headers present on all 6 page types (home, article, about, brand, phase0, 404, feed): X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present.</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr"/>
@@ -4250,7 +4256,7 @@
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: /brand/brand.css?v=brand5 and /img/* both return public,max-age=31536000,immutable; HTML remains public,max-age=0,must-revalidate.</t>
+          <t>PASS — live-verified 2026-08-10: /brand/brand.css?v=brand5 and /img/* both return public,max-age=31536000,immutable; HTML remains public,max-age=0,must-revalidate. | 2026-08-13 re-verified live: versioned assets (/css, /js, /img) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift.</t>
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr"/>
@@ -4462,7 +4468,7 @@
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>PASS — @media (prefers-reduced-motion: reduce) block in tokens.css (loads on every page)</t>
+          <t>PASS — @media (prefers-reduced-motion: reduce) block in tokens.css (loads on every page) | 2026-08-13 re-verified live: verified in the DEPLOYED sheet, not just source: tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, *::before, *::after with !important, plus scroll-behavior auto. Catches all 29 transitioned elements on the homepage.</t>
         </is>
       </c>
       <c r="I78" s="6" t="inlineStr"/>
@@ -4515,7 +4521,7 @@
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-10) — was ISSUE/High: .subscribe-manifesto .sm-submit (homepage + /brand/ subscribe submit) had base and :hover styling but NO :focus-visible rule, so the site's primary conversion control showed no focus indicator for keyboard users (WCAG 2.4.7 AA). Every sibling control was covered — .sm-input directly above it had the rule, and .sm-submit was even named in home-augment.css's prefers-reduced-motion block — so it was an omission, not a decision. Missed by prior runs because F76 was tested at sheet level (':focus-visible present in all 8 stylesheets') rather than per control. Fixed and deployed same day; see p3/p4.</t>
+          <t>PASS (closed live 2026-08-10) — was ISSUE/High: .subscribe-manifesto .sm-submit (homepage + /brand/ subscribe submit) had base and :hover styling but NO :focus-visible rule, so the site's primary conversion control showed no focus indicator for keyboard users (WCAG 2.4.7 AA). Every sibling control was covered — .sm-input directly above it had the rule, and .sm-submit was even named in home-augment.css's prefers-reduced-motion block — so it was an omission, not a decision. Missed by prior runs because F76 was tested at sheet level (':focus-visible present in all 8 stylesheets') rather than per control. Fixed and deployed same day; see p3/p4. | 2026-08-13 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to a footer link that matched ':focus-visible' and computed outline 'solid 2px rgb(204, 0, 0)' at offset 2px.</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
@@ -4572,18 +4578,22 @@
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>PASS — 15 sampled selectors all meet WCAG AA (min 5.17:1 large, 5.94:1 small) in dark mode</t>
-        </is>
-      </c>
-      <c r="I80" s="6" t="inlineStr"/>
+          <t>ISSUE/High (2026-08-13) — .latest-tag (the red 'Latest' chip in the homepage standfirst bar) pairs `background: var(--accent)` with `color: var(--bg)`. In light mode that is cream on #c00 = 5.17:1 and passes. In dark mode --bg flips to #060606 and the same chip computes 3.44:1 at 11.52px/700 — under the 4.5:1 AA floor for small text (WCAG 1.4.3). Measured three times on settled live loads. The #c00/#060606 pair is sanctioned by the Phase 4.1 accent doctrine (DESIGN-SYSTEM.md:102) only for NON-text contrast at the 3:1 floor; this is a text use of it. Missed by prior runs because F77 sampled palette-level token pairs (body/muted/faint/accent text), not the one control that puts small text ON the accent fill — the same sheet-level vs per-control gap that hid F76. All other sampled combinations still pass: 33 distinct fg/bg/size combos in dark, 33 in light, this was the only failure.</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
       <c r="J80" s="4" t="inlineStr">
         <is>
-          <t>NOTE: computed AA: light body 12:1/muted 4.63:1/red 5.34:1; dark body 11.85:1/muted 5.13:1/red 6.2:1; large red 3.44:1&gt;=3</t>
-        </is>
-      </c>
-      <c r="K80" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>FIX (qa/fixes-20260813, commit 549e09c): added `html.dark-mode .issue-latest .latest-tag, html.dark-mode .issue-head .latest-tag { color: var(--ink) }` to css/home-v2.css directly under the base rule. var(--ink) is #f3f0e8 in dark, so the chip renders identically in both modes at 5.17:1. The selector is (0,3,1) and beats the .issue-head hook in home-augment.css (0,2,0) on specificity rather than source order, so only home-v2.css needed the rule and only its cache-bust had to move (?v=phase31 -&gt; phase33 in src/layouts/HomeLayout.astro; the asset is served immutable/1y). brand/index.html needed no edit — it loads home-augment.css but renders no LatestBar.</t>
+        </is>
+      </c>
+      <c r="K80" s="6" t="inlineStr">
+        <is>
+          <t>PASS (build-verified + runtime-verified 2026-08-13, NOT yet live) — `npm run build` clean, 19 pages; dist/index.html references home-v2.css?v=phase33 and dist/css/home-v2.css carries the rule. Cascade verified at runtime on the live DOM: inserting the shipped rule into the real home-v2 sheet via CSSOM insertRule (CSP-safe; a plain &lt;style&gt; injection was blocked by style-src 'self', incidentally reconfirming F69) moved the chip from rgb(6,6,6) to rgb(243,240,232) on rgb(204,0,0) — 3.44:1 -&gt; 5.17:1, passes AA. Goes fully live-verified on the next SCRUB after Dexter merges. Note for merge review: this is a VISIBLE dark-mode change — the chip's word 'Latest' goes from near-black to cream. Light mode is untouched.</t>
         </is>
       </c>
     </row>
@@ -4625,7 +4635,7 @@
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>PASS — single h1 and zero skipped heading levels on all 21 pages; header/main/footer/nav present; zero &lt;img&gt; without alt</t>
+          <t>PASS — single h1 and zero skipped heading levels on all 21 pages; header/main/footer/nav present; zero &lt;img&gt; without alt | 2026-08-13 re-verified live: home and article both single-h1, zero skipped heading levels (home H1 then 17x H2; article H1,H2,H2,H2,H2,H2), header/main/footer/nav all present. Zero images missing alt.</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr"/>
@@ -4731,7 +4741,7 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>PASS — parity 16/16 verified live; every /words/&lt;slug&gt; returns a single 301 to its trailing-slash canonical; no orphan rules</t>
+          <t>PASS — parity 16/16 verified live; every /words/&lt;slug&gt; returns a single 301 to its trailing-slash canonical; no orphan rules | 2026-08-13 re-verified live: all 16 /words/&lt;slug&gt; (no trailing slash) return 301; all 16 /words/&lt;slug&gt;/ return 200 in 0.31-0.45s.</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr"/>
@@ -4852,8 +4862,122 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>F83</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>Dark-mode text on --accent fills (hover treatments)</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>As a dark-mode reader hovering the homepage standfirst bar or the identity-hero primary button, I want the text that inverts onto the red fill to stay readable, so the hover state does not become less legible than the resting state.</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>Every rule that pairs `background: var(--accent)` with small text meets WCAG 1.4.3 in BOTH modes — &gt;=4.5:1 under 18.66px/bold, &gt;=3:1 at or above it.</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>css/home-v2.css:129-135,917-918; css/home-augment.css:146,298</t>
+        </is>
+      </c>
+      <c r="G86" s="6" t="inlineStr">
+        <is>
+          <t>Cataloged 2026-08-13</t>
+        </is>
+      </c>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE/High (2026-08-13) — four hover rules invert small text onto the --accent fill using `color: var(--bg)`, which is #060606 in dark mode = 3.44:1. All four are under their floor: .issue-latest:hover .latest-title (19.2px/400 — NOT large, since AA large needs &gt;=24px or &gt;=18.66px AND bold) 3.44:1; .issue-latest:hover .latest-cta (14.08px/700) 3.44:1; .identity-hero .hero-link.primary:hover (14.08px/700) 3.44:1; and worst, .issue-latest:hover .latest-meta (11.52px/400, hover drops opacity to .6) = 2.54:1. Same root cause as F77 but NOT fixed with it — see p3.</t>
+        </is>
+      </c>
+      <c r="I86" s="6" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="J86" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED — NEEDS DEXTER (fix-phase guardrail: design intent). Unlike F77's resting-state chip, this is a deliberate hover treatment in which the whole standfirst bar inverts to red as one gesture. A colour swap to var(--ink) clears three of the four (5.17:1), but .latest-meta also needs its hover opacity raised off .6 — ink at 60% over #c00 is still only 2.42:1 — and that opacity is a hierarchy decision about how much the meta line should recede, not a defect. Proposed patch held for Dexter's call: `html.dark-mode .issue-latest:hover .latest-title, ...latest-cta, html.dark-mode .identity-hero .hero-link.primary:hover { color: var(--ink) }` plus a decision on the meta's hover opacity.</t>
+        </is>
+      </c>
+      <c r="K86" s="6" t="inlineStr">
+        <is>
+          <t>PENDING — blocked on the design call above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>F84</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Design-system doc &lt;-&gt; implementation parity (accent PROHIBITED-use list)</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>As the owner of the design system, I want the Prohibited accent-use list in DESIGN-SYSTEM.md to match what the CSS actually ships, so the document stays trustworthy as the brand's source of truth.</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>No live rule uses var(--accent) in a way DESIGN-SYSTEM.md:124-130 forbids, or the forbidden entry is annotated with its sanctioned exception.</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>DESIGN-SYSTEM.md:124-130; css/home-v2.css:79-90; css/home-augment.css:93-103</t>
+        </is>
+      </c>
+      <c r="G87" s="6" t="inlineStr">
+        <is>
+          <t>Cataloged 2026-08-13</t>
+        </is>
+      </c>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE/Low (2026-08-13) — DESIGN-SYSTEM.md:124-130 lists 'Backgrounds' and 'Tags or metadata' as PROHIBITED accent uses, but .latest-tag is exactly that: a metadata tag with `background: var(--accent)`, shipped and prominent in the homepage standfirst bar. Companion to F82, which audited only the Permitted half of the same section and so could not have caught this.</t>
+        </is>
+      </c>
+      <c r="I87" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J87" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED — NEEDS DEXTER (fix-phase guardrail: design intent). Two coherent resolutions and the choice is his, exactly as it was for F82: (a) annotate the Prohibited list with the sanctioned exception — the red chip is a deliberate editorial signature and the doc is what is stale; or (b) treat the chip as drift and restyle it. Recommend (a) — the chip reads as authored, and F82's precedent was to correct the doc when the implementation was the considered decision. No CSS touched pending his call. Not deploy-visible either way: /DESIGN-SYSTEM.md returns 404 by design.</t>
+        </is>
+      </c>
+      <c r="K87" s="6" t="inlineStr">
+        <is>
+          <t>PENDING — blocked on the design call above.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:K85"/>
+  <autoFilter ref="A3:K87"/>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A1:K1"/>
@@ -4896,7 +5020,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5">
@@ -4943,7 +5067,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -4960,7 +5084,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -4969,14 +5093,14 @@
           <t>Still open</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>0</v>
+      <c r="B15" s="14" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Total features: 82</t>
+          <t>Total features: 84</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
audit(ledger): close F77 live — Latest chip verified at 5.17:1 on deploy 791bfc5
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -4583,7 +4583,7 @@
       </c>
       <c r="I80" s="6" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGH (closed live)</t>
         </is>
       </c>
       <c r="J80" s="4" t="inlineStr">
@@ -4593,7 +4593,7 @@
       </c>
       <c r="K80" s="6" t="inlineStr">
         <is>
-          <t>PASS (build-verified + runtime-verified 2026-08-13, NOT yet live) — `npm run build` clean, 19 pages; dist/index.html references home-v2.css?v=phase33 and dist/css/home-v2.css carries the rule. Cascade verified at runtime on the live DOM: inserting the shipped rule into the real home-v2 sheet via CSSOM insertRule (CSP-safe; a plain &lt;style&gt; injection was blocked by style-src 'self', incidentally reconfirming F69) moved the chip from rgb(6,6,6) to rgb(243,240,232) on rgb(204,0,0) — 3.44:1 -&gt; 5.17:1, passes AA. Goes fully live-verified on the next SCRUB after Dexter merges. Note for merge review: this is a VISIBLE dark-mode change — the chip's word 'Latest' goes from near-black to cream. Light mode is untouched.</t>
+          <t>PASS (live-verified 2026-08-13, deploy 791bfc5) — merged to main and shipped at Dexter's explicit instruction. Live https://imjustdex.com/ references home-v2.css?v=phase33; the live sheet serves the rule; on the production homepage in dark mode .latest-tag computes rgb(243,240,232) on rgb(204,0,0) at 11.52px/700 = 5.17:1, clearing the 4.5:1 AA floor. Light mode confirmed untouched: rgb(244,244,241) on rgb(204,0,0) = 5.34:1, byte-identical to pre-fix. Post-deploy regression clean — 0 console errors, 16 plates, 3 lane cells, cascade intact. Verification ladder: build-verified 05:50 -&gt; runtime-verified by CSSOM cascade injection 06:05 -&gt; live-verified on production 22:40 CDT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
audit(ledger): close F83/F84 live — accent-fill contrast clear at 5.17:1 on deploy 5c7e5fb
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -63,7 +63,7 @@
       <color rgb="00C0211B"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -88,11 +88,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2E2DE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4B9B5"/>
       </patternFill>
     </fill>
   </fills>
@@ -122,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -147,7 +142,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4915,7 +4909,7 @@
       </c>
       <c r="K86" s="6" t="inlineStr">
         <is>
-          <t>PENDING — awaiting live verification on the deploy.</t>
+          <t>PASS (live-verified 2026-08-13, deploy 5c7e5fb) — verified under REAL pointer hover on the production deploy, in dark mode, with home-v2.css?v=phase34 served. Standfirst bar hovered: .latest-cta now rgb(243,240,232) on rgb(204,0,0) = 5.17:1 (was 3.44:1) PASS; .latest-tag 5.17:1 PASS; .latest-title 17.79:1 PASS; .latest-meta 5.23:1 PASS — all four elements of the hover gesture clear their floor. Identity-hero primary hovered: 'Read the About -&gt;' now rgb(243,240,232) on rgb(204,0,0) = 5.17:1 (was 3.44:1) PASS. Zero console errors post-deploy. No remaining rule on the site pairs small text with the --accent fill below AA in either mode.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4966,7 @@
       </c>
       <c r="K87" s="6" t="inlineStr">
         <is>
-          <t>PENDING — doc-only change; not deploy-visible (/DESIGN-SYSTEM.md returns 404 by design).</t>
+          <t>PASS (2026-08-13, commit 5c7e5fb) — Prohibited-accent list re-read after the edit: the annotation names .latest-tag as the single sanctioned exception, holds the line against further red-filled tags, and states the text-vs-non-text boundary (SC 1.4.3 at 4.5:1 vs Phase 4.1's 3:1 non-text sanction). With F82 (Permitted half) and F84 (Prohibited half) both closed, the full accent section of DESIGN-SYSTEM.md now matches shipped CSS with zero mismatches. Confirmed not deploy-visible: /DESIGN-SYSTEM.md still returns 404. Dexter's 'Two-plane rule' edit verified still present and uncommitted in the working tree after the single-hunk stage.</t>
         </is>
       </c>
     </row>
@@ -5057,7 +5051,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10">
@@ -5067,7 +5061,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -5084,7 +5078,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -5093,8 +5087,8 @@
           <t>Still open</t>
         </is>
       </c>
-      <c r="B15" s="14" t="n">
-        <v>2</v>
+      <c r="B15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
audit(ledger): 2026-08-15 scrub — 84->90 rows, 5 fixed, 1 blocked
F85/F86/F88/F89 opened and fixed (contrast); F87 opened and fixed (the /brand/
dogfood gap); F90 opened BLOCKED — the /brand/ demo-ghost specimens are a
documentation-intent call, not a defect.

F77/F83/F84 p2 normalised to PASS (closed live) to match their p4 and the
F76/F82 convention. F07's `expected` corrected: it claimed articles omit the
feed discovery link, which has not been true since a4f4f25 — the row was
wrong, not the site.

Rotation sample re-verified live: F01, F02, F05, F06, F08-F14.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$3:$K$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$3:$K$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +48,16 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00CC0000"/>
       <sz val="13"/>
     </font>
@@ -63,7 +73,7 @@
       <color rgb="00C0211B"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -87,7 +97,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E0625B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0C24B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A9C7E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E2E2DE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4B9B5"/>
       </patternFill>
     </fill>
   </fills>
@@ -117,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -135,13 +165,26 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -507,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K87"/>
+  <dimension ref="A1:K93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -632,7 +675,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>PASS — masthead .brand-block → '/' present on home/about/404/phase0/brand/article; aria-label 'Dexter Jakes home'</t>
+          <t>PASS — masthead .brand-block → '/' present on home/about/404/phase0/brand/article; aria-label 'Dexter Jakes home' | 2026-08-15 re-verified live: brand-block present and linking / on all 20 pages</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr"/>
@@ -681,7 +724,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>PASS — brand-word: Words (home/article/about/brand), 404, Phase 0 — matches documented intent</t>
+          <t>PASS — brand-word: Words (home/article/about/brand), 404, Phase 0 — matches documented intent | 2026-08-15 re-verified live: brand-word: home/about/article 'Words', 404 '404', phase0 'Phase 0' — matches the documented about-page quirk</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
@@ -836,7 +879,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>PASS — 2 decorative rulers render</t>
+          <t>PASS — 2 decorative rulers render | 2026-08-15 re-verified live: zero .ruler-* without aria-hidden across all pages</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr"/>
@@ -885,7 +928,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>PASS — footer strip + links present on all page types</t>
+          <t>PASS — footer strip + links present on all page types | 2026-08-15 re-verified live: footer: Instagram + X both target=_blank rel="noopener noreferrer", /feed.xml, /about/, "Built by Dex"; zero _blank links missing rel site-wide</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
@@ -919,7 +962,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>&lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in &lt;head&gt; on home, about, phase0. (Articles/coming-soon/404 do NOT include it — verify intent.)</t>
+          <t>&lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in &lt;head&gt; on home, about, phase0 AND articles (ArticleLayout.astro:123 — added at commit a4f4f25). 404 does NOT include it (noindex page).</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -934,7 +977,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>PASS — &lt;link rel=alternate atom&gt; present on home, about, phase0, article</t>
+          <t>PASS (2026-08-15 scrub) — home/about/phase0/articles all carry the feed discovery link; /404 correctly omits it. NOTE: the prior `expected` said articles do NOT include it. That text was stale — ArticleLayout has emitted the link since a4f4f25; the site was never wrong, the row was. Expectation corrected, not the code.</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr"/>
@@ -987,7 +1030,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>PASS — /img/favicon-32.png + /img/apple-touch-icon.png 200 on every referenced path | 2026-08-13 re-verified live: /img/favicon-32.png and /img/apple-touch-icon.png both 200, immutable-cached.</t>
+          <t>PASS — /img/favicon-32.png + /img/apple-touch-icon.png 200 on every referenced path | 2026-08-15 re-verified live: favicon-32.png + apple-touch-icon.png linked on every page; both 200 (1327b / 5729b)</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr"/>
@@ -1036,7 +1079,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>PASS — Anton + IBM Plex Sans self-hosted, preloaded, document.fonts status 'loaded'; CSP font-src intact | 2026-08-13 re-verified live: document.fonts.status 'loaded'; Anton 400, IBM Plex Sans 400 + 700 all report 'loaded' on home and article. No FOUT observed.</t>
+          <t>PASS — Anton + IBM Plex Sans self-hosted, preloaded, document.fonts status 'loaded'; CSP font-src intact | 2026-08-15 re-verified live: Anton + IBM Plex Sans preloaded with crossorigin; zero Google Fonts refs; document.fonts reports all 3 faces loaded</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr"/>
@@ -1085,7 +1128,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>PASS — no horizontal overflow at 390px on home/article/about/phase0/brand/404</t>
+          <t>PASS — no horizontal overflow at 390px on home/article/about/phase0/brand/404 | 2026-08-15 re-verified live: viewport width=device-width + viewport-fit=cover on all pages</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
@@ -1138,7 +1181,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>PASS — title/description/canonical on all 21 routes; every canonical on imjustdex.com | 2026-08-13 re-verified live: title/description/canonical present and pointing at imjustdex.com on all 16 articles + home/about/brand/phase0.</t>
+          <t>PASS — title/description/canonical on all 21 routes; every canonical on imjustdex.com | 2026-08-15 re-verified live: zero duplicate &lt;title&gt; across 20 pages; /404 canonical is /404 as specified</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr"/>
@@ -1187,7 +1230,7 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>PASS — og+twitter complete on all 21; all 19 OG images 200 (16 essays + home/about/phase0/brand) | 2026-08-13 re-verified live: og:title/og:description/og:image/twitter:card present on all 16 articles; og:image matches the JSON-LD image URL exactly (same cache-bust) on every one.</t>
+          <t>PASS — og+twitter complete on all 21; all 19 OG images 200 (16 essays + home/about/phase0/brand) | 2026-08-15 re-verified live: twitter:card summary_large_image on every page in scope (404 correctly excluded)</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr"/>
@@ -1240,7 +1283,7 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>PASS — WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor) | 2026-08-13 re-verified live: homepage @graph carries WebSite + Person; Person has all of name/url/sameAs/jobTitle/worksFor.</t>
+          <t>PASS — WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor) | 2026-08-15 re-verified live: home @graph carries WebSite + Person; Person has name/url/sameAs/jobTitle/worksFor — no missing fields</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr"/>
@@ -1289,7 +1332,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>PASS — ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description) | 2026-08-13 re-verified live: /about/ ProfilePage mainEntity is @type Person with name/url/jobTitle/worksFor/sameAs/description — zero missing fields.</t>
+          <t>PASS — ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description) | 2026-08-15 re-verified live: about ProfilePage mainEntity Person complete — name/url/jobTitle/worksFor/sameAs/description all present</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
@@ -4572,12 +4615,12 @@
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-13) — .latest-tag (the red 'Latest' chip in the homepage standfirst bar) pairs `background: var(--accent)` with `color: var(--bg)`. In light mode that is cream on #c00 = 5.17:1 and passes. In dark mode --bg flips to #060606 and the same chip computes 3.44:1 at 11.52px/700 — under the 4.5:1 AA floor for small text (WCAG 1.4.3). Measured three times on settled live loads. The #c00/#060606 pair is sanctioned by the Phase 4.1 accent doctrine (DESIGN-SYSTEM.md:102) only for NON-text contrast at the 3:1 floor; this is a text use of it. Missed by prior runs because F77 sampled palette-level token pairs (body/muted/faint/accent text), not the one control that puts small text ON the accent fill — the same sheet-level vs per-control gap that hid F76. All other sampled combinations still pass: 33 distinct fg/bg/size combos in dark, 33 in light, this was the only failure.</t>
+          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — .latest-tag (the red 'Latest' chip in the homepage standfirst bar) pairs `background: var(--accent)` with `color: var(--bg)`. In light mode that is cream on #c00 = 5.17:1 and passes. In dark mode --bg flips to #060606 and the same chip computes 3.44:1 at 11.52px/700 — under the 4.5:1 AA floor for small text (WCAG 1.4.3). Measured three times on settled live loads. The #c00/#060606 pair is sanctioned by the Phase 4.1 accent doctrine (DESIGN-SYSTEM.md:102) only for NON-text contrast at the 3:1 floor; this is a text use of it. Missed by prior runs because F77 sampled palette-level token pairs (body/muted/faint/accent text), not the one control that puts small text ON the accent fill — the same sheet-level vs per-control gap that hid F76. All other sampled combinations still pass: 33 distinct fg/bg/size combos in dark, 33 in light, this was the only failure.</t>
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr">
         <is>
-          <t>HIGH (closed live)</t>
+          <t>HIGH (closed live) (resolved)</t>
         </is>
       </c>
       <c r="J80" s="4" t="inlineStr">
@@ -4894,12 +4937,12 @@
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-13) — CORRECTED SCOPE, and the correction matters. The morning scrub read the declarations and reported FOUR failing hover rules. Re-measured under REAL pointer hover before fixing, only TWO are real: `.issue-latest:hover .latest-cta` (14.08px/700) and `.identity-hero .hero-link.primary:hover` (14.08px/700), both `color: var(--bg)` on a `background: var(--accent)` fill = 3.44:1 in dark against a 4.5:1 floor. The other two were FALSE POSITIVES: `.issue-latest:hover` takes the BAR to var(--ink), not var(--accent), so .latest-title measures 17.79:1 and .latest-meta 5.23:1 (at opacity .6) against cream — both already clear. The morning read assumed the accent fill was the surface for every child of the hover state; it is only the surface for .latest-cta, which sets its own background. Lesson: resolve the PAINTED surface under real hover, never infer it from the parent's declarations.</t>
+          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — CORRECTED SCOPE, and the correction matters. The morning scrub read the declarations and reported FOUR failing hover rules. Re-measured under REAL pointer hover before fixing, only TWO are real: `.issue-latest:hover .latest-cta` (14.08px/700) and `.identity-hero .hero-link.primary:hover` (14.08px/700), both `color: var(--bg)` on a `background: var(--accent)` fill = 3.44:1 in dark against a 4.5:1 floor. The other two were FALSE POSITIVES: `.issue-latest:hover` takes the BAR to var(--ink), not var(--accent), so .latest-title measures 17.79:1 and .latest-meta 5.23:1 (at opacity .6) against cream — both already clear. The morning read assumed the accent fill was the surface for every child of the hover state; it is only the surface for .latest-cta, which sets its own background. Lesson: resolve the PAINTED surface under real hover, never infer it from the parent's declarations.</t>
         </is>
       </c>
       <c r="I86" s="6" t="inlineStr">
         <is>
-          <t>HIGH (closed live)</t>
+          <t>HIGH (closed live) (resolved)</t>
         </is>
       </c>
       <c r="J86" s="4" t="inlineStr">
@@ -4951,12 +4994,12 @@
       </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-08-13) — DESIGN-SYSTEM.md:124-130 lists 'Backgrounds' and 'Tags or metadata' as PROHIBITED accent uses, but .latest-tag is exactly that: a metadata tag with `background: var(--accent)`, shipped and prominent in the homepage standfirst bar. Companion to F82, which audited only the Permitted half of the same section and so could not have caught this.</t>
+          <t>PASS (closed live 2026-08-13) — was ISSUE/Low (2026-08-13) — DESIGN-SYSTEM.md:124-130 lists 'Backgrounds' and 'Tags or metadata' as PROHIBITED accent uses, but .latest-tag is exactly that: a metadata tag with `background: var(--accent)`, shipped and prominent in the homepage standfirst bar. Companion to F82, which audited only the Permitted half of the same section and so could not have caught this.</t>
         </is>
       </c>
       <c r="I87" s="6" t="inlineStr">
         <is>
-          <t>LOW (closed live)</t>
+          <t>LOW (closed live) (resolved)</t>
         </is>
       </c>
       <c r="J87" s="4" t="inlineStr">
@@ -4970,8 +5013,350 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>F85</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>Standfirst metadata contrast (--body-muted + opacity multiplier)</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>As a reader on either mode, I can read the lane/date/read-time metadata in the homepage standfirst bar.</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>Text using var(--body-muted) meets WCAG 1.4.3 (&gt;=4.5:1 at this 11.52px/400 size) in BOTH modes. The token is alpha-tuned to clear the floor on its own; no rule may stack a second opacity multiplier on top of it.</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>css/home-v2.css:112-122; css/home-augment.css:119-129; src/components/home/LatestBar.astro:27</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>Cataloged</t>
+        </is>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE/High (2026-08-15) — `.latest-meta` ('Faith · Jul 5 · 16 min', the metadata in the homepage standfirst bar) pairs `color: var(--body-muted)` with `opacity: .75`. --body-muted is ALREADY an alpha colour (rgba(243,240,232,.52) dark / rgba(5,5,5,.56) light), tuned to land just over AA on its own — 5.13:1 dark, 4.67:1 light. The extra multiplier composites a second time and drops the control to 3.36:1 dark / 2.93:1 light, under the 4.5:1 floor for 11.52px/400 text. FAILS IN BOTH MODES — the only finding this run that is not dark-mode-specific. Measured on the settled live page with a compositor that resolves the painted surface by walking every ancestor background (flat #0d0d0d here, no image layer to confound it), then confirmed visually in a full-page screenshot where this is plainly the faintest text on the homepage. Missed by every prior run for a precise reason: the 2026-08-13 scrub measured .latest-meta ONLY under pointer hover, where `.issue-latest:hover .latest-meta` re-declares `color: var(--bg); opacity: .6` against the cream hover bar and clears at 5.23:1. F83 recorded that number and closed the question. The RESTING state — which is what a reader actually sees — was never measured.</t>
+        </is>
+      </c>
+      <c r="I88" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J88" s="4" t="inlineStr">
+        <is>
+          <t>FIX (qa/fixes-20260815): deleted `opacity: .75` from both `.issue-latest .latest-meta` (css/home-v2.css) and `.issue-head .latest-meta` (css/home-augment.css), leaving var(--body-muted) to carry the muting alone. Both sheets edited because both paint this control (home-v2 wins on the homepage by source order; home-augment is the sheet /brand/ loads). Comment left in both explaining that the token IS the muted level. The hover rules were deliberately left untouched — they set their own opacity and already measured 5.23:1. Cache-bust bumped home-augment phase32-&gt;phase33, home-v2 phase34-&gt;phase35 (both sheets ship immutable/1yr).</t>
+        </is>
+      </c>
+      <c r="K88" s="6" t="inlineStr">
+        <is>
+          <t>PASS (build-verified 2026-08-15) — `npm run build` clean, 19 pages. dist/css/*.css confirmed to carry the rules with zero opacity declarations. Post-fix values measured on the live DOM with the exact shipped declarations applied: dark 3.36:1 -&gt; 5.13:1, light 2.93:1 -&gt; 4.67:1. Both clear the 4.5:1 floor. Goes live-verified on the next scrub after Dexter merges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>F86</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>Identity-hero corner label contrast (dark mode)</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>As a reader in dark mode, I can read the 'The Writer → 01' corner label on the identity hero.</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>`.identity-hero .hero-corner` meets WCAG 1.4.3 (&gt;=4.5:1 at 11.52px/700) in both modes, on whichever ground the hero plate presents.</t>
+        </is>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>css/home-augment.css:185-200; css/home-v2.css:864-878; src/components/home/IdentityHero.astro:7</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>Cataloged</t>
+        </is>
+      </c>
+      <c r="H89" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE/High (2026-08-15) — `.hero-corner` sets `color: var(--bg); opacity: .5`. The identity hero is an INVERTED plate: in dark mode it presents a cream ground (243,240,232) and the label paints #060606 over it, which at .5 opacity computes 3.71:1 — under the 4.5:1 floor for 11.52px/700 (bold, but well below the 18.66px large-text threshold). Light mode inverts to cream-on-black and clears at 4.91:1, so this is dark-mode-only. Same root shape as F85 — a decorative opacity multiplier stacked on a colour that was already correct — but reached by the opposite route: here the multiplier sits on a SOLID token rather than an alpha one. Surface resolved by walking to the first opaque ancestor (.hero-main, flat cream, no image layer); confirmed visually in a dark-mode full-page screenshot.</t>
+        </is>
+      </c>
+      <c r="I89" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J89" s="4" t="inlineStr">
+        <is>
+          <t>FIX (qa/fixes-20260815): raised `opacity: .5` -&gt; `.6` on `.identity-hero .hero-corner` in both css/home-augment.css and css/home-v2.css. The value is not arbitrary: the computed minimum to clear 4.5:1 on this pair is .56, solved by stepping opacity in 0.005 increments against the real painted ground; .6 takes it clear with margin while keeping the label recessive. Removing the multiplier entirely was rejected — that would be 17.79:1, a visual change to the hero's balance rather than a contrast repair.</t>
+        </is>
+      </c>
+      <c r="K89" s="6" t="inlineStr">
+        <is>
+          <t>PASS (build-verified 2026-08-15) — post-fix values measured on the live DOM with opacity .6 applied: dark 3.71:1 -&gt; 5.23:1, light 4.91:1 -&gt; 6.74:1. Both clear. dist confirmed to carry `opacity: .6` in both sheets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>F87</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>/brand/ dogfood contract — shared-component fixes must land in the shared sheet</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>As the design system's own documentation, /brand/ renders production classes and therefore shows exactly what the live site shows — including fixes.</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>Any fix to a component that /brand/ demos must live in a stylesheet /brand/ actually loads (tokens, shell, plates, home-augment, article — NOT home-v2.css, which is homepage-only).</t>
+        </is>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>brand/index.html:39,115; css/home-augment.css; css/home-v2.css</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>Cataloged</t>
+        </is>
+      </c>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE/High (2026-08-15) — /brand/ was still rendering `.latest-tag` at 3.44:1, the exact pre-fix value F77 closed on 2026-08-13, two days after that row went green. Cause: the F77 and F83 dark-mode overrides were written into css/home-v2.css. The homepage loads home-augment.css AND home-v2.css; /brand/ loads home-augment.css and never home-v2.css. So the fixes reached the homepage and silently skipped the design system's own documentation page. This is a broken contract, not a cosmetic gap: brand/index.html:115 states a 'Dogfood rule' — '/brand/ runs the same stylesheets as the live site... If a live component breaks, this page breaks too. That is intentional.' A fix that lands on one surface and not the other makes the dogfood page a liar in the safer direction, which is worse than an obvious break. The F77 comment even asserted it 'Covers the .issue-head hook in home-augment.css too; wins on specificity, not source order' — true about specificity, but specificity is irrelevant in a sheet that never loads.</t>
+        </is>
+      </c>
+      <c r="I90" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J90" s="4" t="inlineStr">
+        <is>
+          <t>FIX (qa/fixes-20260815): moved both override blocks — `html.dark-mode .issue-latest .latest-tag, html.dark-mode .issue-head .latest-tag` [F77] and `html.dark-mode .issue-latest:hover .latest-cta, html.dark-mode .identity-hero .hero-link.primary:hover` [F83] — out of css/home-v2.css and into css/home-augment.css, the sheet both surfaces load. Breadcrumb comments left at both former sites in home-v2.css so the next reader finds them. The relocation is cascade-safe and was verified as such rather than assumed: the overrides are (0,3,1), (0,4,1) and (0,5,1) against base rules of (0,2,0), (0,3,0) and (0,4,0), so they win on specificity and source order cannot take them back — which is why moving them EARLIER in the cascade is safe.</t>
+        </is>
+      </c>
+      <c r="K90" s="6" t="inlineStr">
+        <is>
+          <t>PASS (build-verified 2026-08-15) — grepped the built sheets: dist/css/home-augment.css carries both blocks at lines 127-134, dist/css/home-v2.css carries neither (only the breadcrumbs). Measured on the live /brand/ page in dark mode with the override applied: `.latest-tag` 3.44:1 -&gt; 5.17:1, the identical figure the homepage has been serving since deploy 791bfc5. Dogfood parity restored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>F88</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Homepage</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>Issue-next strip metadata contrast (latent)</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>As a reader, when an upcoming essay is scheduled I can read the Issue-next strip's lane/date/read-time metadata.</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>`.issue-next .next-meta` meets WCAG 1.4.3 (&gt;=4.5:1 at 11.52px/400) in both modes whenever the Issue-next strip renders.</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>css/home-v2.css:220-230; css/home-augment.css:691-701; src/components/home/IssueNext.astro:20</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>Cataloged</t>
+        </is>
+      </c>
+      <c r="H91" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE/Medium (2026-08-15) — `.next-meta` repeats the F85 defect one notch worse: `color: var(--body-muted)` plus `opacity: .65`, computing 2.81:1 in dark against the 4.5:1 floor. Graded MEDIUM rather than HIGH because it is LATENT — the Issue-next strip only renders when an upcoming essay exists, and all 16 entries are status:published with past dates (see F41/F46), so no reader has hit it. It was found because /brand/ demos the strip under its dogfood rule, which is the same page that exposed F87. Worth recording precisely: this would have shipped broken on the day Dexter scheduled his next essay, and it would have shipped inside the one component whose whole job is to advertise that essay.</t>
+        </is>
+      </c>
+      <c r="I91" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J91" s="4" t="inlineStr">
+        <is>
+          <t>FIX (qa/fixes-20260815): deleted `opacity: .65` from `.issue-next .next-meta` in both css/home-v2.css and css/home-augment.css, same treatment and same reasoning as F85.</t>
+        </is>
+      </c>
+      <c r="K91" s="6" t="inlineStr">
+        <is>
+          <t>PASS (build-verified 2026-08-15) — measured on the live /brand/ demo of the strip in dark mode with the fix applied: 2.81:1 -&gt; 5.13:1. Clears. (An earlier reading of 1.02:1 during this run was an artifact of forcing the dark-mode class onto an already-rendered light page, which left tokens half-resolved; discarded and re-measured after a clean reload with the dxmode cookie set. Recording it here so the number is not mistaken for a real regression if it resurfaces.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>F89</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>404 eyebrow divider contrast</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>As a reader landing on a bad URL, I can read the eyebrow strip 'ERROR · 404 · PAGE NOT FOUND' in full.</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>`.notfound-eyebrow span.divider` meets WCAG 1.4.3, or is marked aria-hidden and treated as decoration.</t>
+        </is>
+      </c>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>css/notfound.css:64-66; src/pages/404.astro</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>Cataloged</t>
+        </is>
+      </c>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE/Medium (2026-08-15) — the `·` separators in the 404 eyebrow carry `opacity: .5`, computing 3.61:1. Unlike the homepage's `.dot` separators — which are `aria-hidden="true"` and therefore exempt as decoration — these carry no aria-hidden, so they are exposed text in both the accessibility tree and the visual read. Caught by explicitly checking aria-hidden per separator rather than assuming all separators are decorative: the homepage `.dot` at 4.25:1 was correctly DISMISSED as a non-finding by that same check, and this one was correctly kept.</t>
+        </is>
+      </c>
+      <c r="I92" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J92" s="4" t="inlineStr">
+        <is>
+          <t>FIX (qa/fixes-20260815): raised `opacity: .5` -&gt; `.7` in css/notfound.css. Value taken from the file's own convention — the adjacent `.notfound-eyebrow .eyebrow-right` rule already uses .7 — rather than inventing a number. Cache-bust bumped notfound.css phase10 -&gt; phase11 in src/pages/404.astro.</t>
+        </is>
+      </c>
+      <c r="K92" s="6" t="inlineStr">
+        <is>
+          <t>PASS (build-verified 2026-08-15) — measured on the live /404 with opacity .7 applied: 3.61:1 -&gt; 7.19:1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>/brand/ bespoke + demo-specimen contrast (documentation surface)</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>As a reader of the design system doc, I can read its bespoke chrome and its component specimens.</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>Text on /brand/ meets WCAG 1.4.3, or the recessive treatment is a deliberate demonstration and is recorded as such.</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>brand/brand.css; brand/index.html (demo-ghost-*, Download Pack h3)</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>Cataloged</t>
+        </is>
+      </c>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE/Low (2026-08-15) — five /brand/-only text elements measure under AA in dark mode: `.demo-ghost-meta` ('Coming Soon') 2.05:1, `.demo-ghost-date` 2.45:1, `.demo-ghost-title` 2.93:1 (against its 3:1 large-text floor), `.demo-plate-meta` 3.17:1, and the bespoke 'Download Pack' h3 at 2.87:1. Held BLOCKED rather than fixed: four of the five are `demo-ghost-*` specimens whose entire purpose is to DEMONSTRATE the dim 'not yet published' ghost treatment, so raising their contrast would edit the documentation's illustration rather than repair a defect — that is a call about what the design system wants to say, and it is Dexter's. The fifth ('Download Pack') is bespoke brand.css chrome and is a genuine, if low-traffic, AA miss. Deliberately NOT bundled with F87: that row was a broken contract with an objectively correct fix; this one is a judgement about intent.</t>
+        </is>
+      </c>
+      <c r="I93" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J93" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED — NEEDS DEXTER. Two questions: (a) should the ghost specimens keep their dim demonstration value, or does the doc need a readable annotation beside them explaining the treatment? (b) the "Download Pack" h3 in brand.css is not a specimen and can be lifted on his word.</t>
+        </is>
+      </c>
+      <c r="K93" s="6" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:K87"/>
+  <autoFilter ref="A3:K93"/>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A1:K1"/>
@@ -4986,7 +5371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4994,14 +5379,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Phase 2 Test Results</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>— P2 (test) —</t>
         </is>
@@ -5013,8 +5398,8 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="B4" s="9" t="n">
-        <v>77</v>
+      <c r="B4" s="12" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="5">
@@ -5023,7 +5408,7 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5033,12 +5418,12 @@
           <t>PENDING</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="14" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>— P4 (re-test) —</t>
         </is>
@@ -5050,8 +5435,8 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n">
-        <v>81</v>
+      <c r="B9" s="12" t="n">
+        <v>86</v>
       </c>
     </row>
     <row r="10">
@@ -5060,41 +5445,71 @@
           <t>PENDING</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>— Issues by severity (found) —</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>— Issues by severity (found) —</t>
-        </is>
-      </c>
-    </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>Resolved (P4 PASS)</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="B17" s="12" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>Still open</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Total features: 84</t>
+      <c r="B18" s="20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Total features: 90</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
audit(ledger): F93 fixed — ghost plate rewired, verified on a fixture build
Dexter chose rewire over retire. Records the three decisions (static per the
doc; head-of-cascade placement to preserve reverse chronology; no data-lane so
lane filters hide it and the published-only counts stay honest) and the full
fixture verification.

Side effect worth noting: the plates.css half of the F90 fix is no longer
unverifiable. The ghost plate has an emitter now, and on the fixture build its
title/date/meta/lane measured 3.40/5.11/5.11/5.11 dark and 3.31/4.62/4.62/4.62
light — the values F90 predicted.

Observed but not opened as its own row: DESIGN-SYSTEM.md specifies .plate-ghost
min-height 346px, plates.css ships 230px. Doc-vs-implementation drift of the
F82/F84 class, but that file carries Dexter's uncommitted "Two-plane rule"
edit, so reconciling it is his, not the loop's.

F73 is now the only open row across 93.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -5488,22 +5488,22 @@
       </c>
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-08-27) — both class names are DEAD in production. `Plate.astro` can only ever emit `plate plate-{wide|secondary|banner|half|lead}` plus `plate-image`, `img-*` and `plate-row`; there is no code path to `plate-ghost` or `identity-plate`, the strings appear nowhere in src/, and they appear in none of the 19 built pages. This is almost certainly fallout from the 2026-04-21 Astro cutover — the ghost teaser is clearly still intended (ComingSoonLayout exists, visibility.ts date-gates future essays, and F30/F41 both describe an upcoming-essay flow), it just never got rewired to the new cascade. Two consequences: css/plates.css ships ~90 lines of unreachable rules on every homepage load, and /brand/ documents both as live components when neither can render. Found while re-diagnosing F90 — the F90 contrast failures are in these same dead rules, which is why they only ever surfaced on /brand/.</t>
-        </is>
-      </c>
-      <c r="I96" s="7" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>ISSUE/Medium (2026-08-27) — both class names are DEAD in production. `Plate.astro` can only ever emit `plate plate-{wide|secondary|banner|half|lead}` plus `plate-image`, `img-*` and `plate-row`; there is no code path to `plate-ghost` or `identity-plate`, the strings appear nowhere in src/, and they appear in none of the 19 built pages. This is almost certainly fallout from the 2026-04-21 Astro cutover — the ghost teaser is clearly still intended (ComingSoonLayout exists, visibility.ts date-gates future essays, and F30/F41 both describe an upcoming-essay flow), it just never got rewired to the new cascade. Two consequences: css/plates.css ships ~90 lines of unreachable rules on every homepage load, and /brand/ documents both as live components when neither can render. Found while re-diagnosing F90 — the F90 contrast failures are in these same dead rules, which is why they only ever surfaced on /brand/. | Dexter chose REWIRE over retire, 2026-08-27.</t>
+        </is>
+      </c>
+      <c r="I96" s="6" t="inlineStr">
+        <is>
+          <t>Medium (fixed)</t>
         </is>
       </c>
       <c r="J96" s="4" t="inlineStr">
         <is>
-          <t>BLOCKED — NEEDS DEXTER. Not auto-fixable in either direction: rewiring the ghost plate into the cascade is a layout/product decision (where an upcoming essay sits in the reading order, whether it counts in the lane index, whether it is linkable), and deleting the rules retires two documented components from the design system. Both are your call. The contrast fix from F90 is already applied to these rules either way, so whichever direction you pick, they ship AA-clean.</t>
+          <t>FIX (qa/fixes-20260827, 96b0bc9) — new src/components/home/GhostPlate.astro emits the held-space card for every isUpcoming entry, wired into src/pages/index.astro as its own '01 / Next' section at the head of the cascade. Three decisions, all taken from DESIGN-SYSTEM.md rather than invented: (1) STATIC — no &lt;a&gt;, no href, no hover, no focus ring, per the doc's 'identity plate, ghost teaser (static). No hover highlight, no pointer cursor, no focus outline'; the linked CTA for the same essay remains the IssueNext strip, so the plate holds the space and the strip does the asking. (2) PLACEMENT at the head of the cascade — the cascade's organising principle is strict reverse chronology and an upcoming essay is newer than the lead, so this is the only placement that preserves it; at span 5 the ghost does not dominate and the lead plate's full-width hero sits immediately beneath. (3) NO data-lane, which is load-bearing: lane-filter.js matches on the inner [data-lane], so with none the ghost is hidden by any active filter and restored by baseHidden() on clear — keeping the published-only lane counts (F22) honest against what is on screen. Row-head numbers were hardcoded 01/02 plus a conditional on Earlier, which cannot survive a section appearing above them; now derived from which sections actually render.</t>
         </is>
       </c>
       <c r="K96" s="6" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>PASS (verified against build) — 2026-08-27. The collection holds no upcoming entry, so verification used a temporary future-dated fixture, removed before commit (git status clean of it). Renders span 5 at 503x230 desktop, span 1 at 339px mobile with no overflow at 375px. Static: cursor default, not a link, not focusable. Contrast clears AA on the values F90 just landed — title 3.40 dark / 3.31 light (floor 3.0); teaser-date, meta rail and lane badge all 5.11 dark / 4.62 light (floor 4.5). Single h1, no skipped heading levels. Lane filter: 9 visible with ghost -&gt; Faith 13 ghost hidden -&gt; clear 9 ghost back -&gt; Art 3 ghost hidden (matching the lane index exactly) -&gt; clear 9. Earlier toggle: expand 17 / collapse 9, glyph tracks, ghost unaffected. With zero upcoming the page is behaviourally identical to before — row heads 01/02/03, no ghost markup. Zero console errors in both modes. Does not surface Dexter's before-i-had-the-words.mdx (status 'drafted' fails isUpcomingData). OBSERVED, not opened as its own row: DESIGN-SYSTEM.md specifies .plate-ghost min-height 346px while plates.css ships 230px. Doc-vs-implementation drift of the F82/F84 class, but the doc file currently carries Dexter's uncommitted 'Two-plane rule' edit, so it is his to reconcile, not the loop's.</t>
         </is>
       </c>
     </row>
@@ -5588,7 +5588,7 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10">
@@ -5598,7 +5598,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -5615,7 +5615,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -5625,7 +5625,7 @@
         </is>
       </c>
       <c r="B15" s="10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
@@ -5635,7 +5635,7 @@
         </is>
       </c>
       <c r="B16" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
audit(ledger): F93 shipped on 2387e1d — verified inert until an essay is scheduled
The ghost plate cannot be observed on production yet: the collection holds no
upcoming entry. So what was verified live is that the change is INERT until one
exists, which is the correct outcome —

  row heads   01 This Week / 02 This Month / 03 Earlier (unchanged)
  ghost       0 .plate-ghost in the DOM
  IssueNext   correctly absent (F30)
  cascade     16 plates; filter Faith 13, clear 8; toggle 8<->16, glyph tracks
  console     clean
  sweep       25 routes 200, both 404s, 5/5 headers, feed 16, sitemap 20 locs

The rendering and the section renumbering were verified pre-push on a fixture
build. They will first be exercised on production the day an essay is
scheduled; the next SCRUB after that should re-test F93 and F30 live.

End of day: 93 rows, one open — F73, the GitHub cron, not a site defect.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -5488,7 +5488,7 @@
       </c>
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-08-27) — both class names are DEAD in production. `Plate.astro` can only ever emit `plate plate-{wide|secondary|banner|half|lead}` plus `plate-image`, `img-*` and `plate-row`; there is no code path to `plate-ghost` or `identity-plate`, the strings appear nowhere in src/, and they appear in none of the 19 built pages. This is almost certainly fallout from the 2026-04-21 Astro cutover — the ghost teaser is clearly still intended (ComingSoonLayout exists, visibility.ts date-gates future essays, and F30/F41 both describe an upcoming-essay flow), it just never got rewired to the new cascade. Two consequences: css/plates.css ships ~90 lines of unreachable rules on every homepage load, and /brand/ documents both as live components when neither can render. Found while re-diagnosing F90 — the F90 contrast failures are in these same dead rules, which is why they only ever surfaced on /brand/. | Dexter chose REWIRE over retire, 2026-08-27.</t>
+          <t>ISSUE/Medium (2026-08-27) — both class names are DEAD in production. `Plate.astro` can only ever emit `plate plate-{wide|secondary|banner|half|lead}` plus `plate-image`, `img-*` and `plate-row`; there is no code path to `plate-ghost` or `identity-plate`, the strings appear nowhere in src/, and they appear in none of the 19 built pages. This is almost certainly fallout from the 2026-04-21 Astro cutover — the ghost teaser is clearly still intended (ComingSoonLayout exists, visibility.ts date-gates future essays, and F30/F41 both describe an upcoming-essay flow), it just never got rewired to the new cascade. Two consequences: css/plates.css ships ~90 lines of unreachable rules on every homepage load, and /brand/ documents both as live components when neither can render. Found while re-diagnosing F90 — the F90 contrast failures are in these same dead rules, which is why they only ever surfaced on /brand/. | Dexter chose REWIRE over retire, 2026-08-27. | RESOLVED 2026-08-27 — see p4.</t>
         </is>
       </c>
       <c r="I96" s="6" t="inlineStr">
@@ -5503,7 +5503,7 @@
       </c>
       <c r="K96" s="6" t="inlineStr">
         <is>
-          <t>PASS (verified against build) — 2026-08-27. The collection holds no upcoming entry, so verification used a temporary future-dated fixture, removed before commit (git status clean of it). Renders span 5 at 503x230 desktop, span 1 at 339px mobile with no overflow at 375px. Static: cursor default, not a link, not focusable. Contrast clears AA on the values F90 just landed — title 3.40 dark / 3.31 light (floor 3.0); teaser-date, meta rail and lane badge all 5.11 dark / 4.62 light (floor 4.5). Single h1, no skipped heading levels. Lane filter: 9 visible with ghost -&gt; Faith 13 ghost hidden -&gt; clear 9 ghost back -&gt; Art 3 ghost hidden (matching the lane index exactly) -&gt; clear 9. Earlier toggle: expand 17 / collapse 9, glyph tracks, ghost unaffected. With zero upcoming the page is behaviourally identical to before — row heads 01/02/03, no ghost markup. Zero console errors in both modes. Does not surface Dexter's before-i-had-the-words.mdx (status 'drafted' fails isUpcomingData). OBSERVED, not opened as its own row: DESIGN-SYSTEM.md specifies .plate-ghost min-height 346px while plates.css ships 230px. Doc-vs-implementation drift of the F82/F84 class, but the doc file currently carries Dexter's uncommitted 'Two-plane rule' edit, so it is his to reconcile, not the loop's.</t>
+          <t>PASS (verified against build) — 2026-08-27. The collection holds no upcoming entry, so verification used a temporary future-dated fixture, removed before commit (git status clean of it). Renders span 5 at 503x230 desktop, span 1 at 339px mobile with no overflow at 375px. Static: cursor default, not a link, not focusable. Contrast clears AA on the values F90 just landed — title 3.40 dark / 3.31 light (floor 3.0); teaser-date, meta rail and lane badge all 5.11 dark / 4.62 light (floor 4.5). Single h1, no skipped heading levels. Lane filter: 9 visible with ghost -&gt; Faith 13 ghost hidden -&gt; clear 9 ghost back -&gt; Art 3 ghost hidden (matching the lane index exactly) -&gt; clear 9. Earlier toggle: expand 17 / collapse 9, glyph tracks, ghost unaffected. With zero upcoming the page is behaviourally identical to before — row heads 01/02/03, no ghost markup. Zero console errors in both modes. Does not surface Dexter's before-i-had-the-words.mdx (status 'drafted' fails isUpcomingData). OBSERVED, not opened as its own row: DESIGN-SYSTEM.md specifies .plate-ghost min-height 346px while plates.css ships 230px. Doc-vs-implementation drift of the F82/F84 class, but the doc file currently carries Dexter's uncommitted 'Two-plane rule' edit, so it is his to reconcile, not the loop's. || SHIPPED LIVE 2026-08-27 on deploy 2387e1d. The ghost plate cannot be observed on production yet — the collection holds no upcoming entry — so what was verified live is that the change is INERT until one exists, which is the correct behaviour: row heads read 01 This Week / 02 This Month / 03 Earlier, zero .plate-ghost markup, IssueNext correctly absent (F30), 16 plates, lane filter Faith 13 and clear back to 8, earlier toggle 8&lt;-&gt;16 with the glyph tracking, zero console errors. Sweep clean: 25 routes 200, both correct 404s, 5/5 security headers, feed 16 entries, sitemap 20 locs. The section-numbering and ghost rendering will first be exercised on production the day Dexter schedules an essay; that run's SCRUB should re-test this row live.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
audit(ledger): F30 -> N/A, F94 records the completed retirement
F30's component no longer exists, so the row goes N/A per the never-delete
rule. Future runs must not test it and must not flag the strip's absence — but
SHOULD flag it if `.issue-next` ever reappears in the DOM or in any shipped
stylesheet, which would mean the retirement regressed.

F94 carries the full record: what was removed, why /brand/ needed a retirement
note rather than a delete, and the verification.

Carried forward: DESIGN-SYSTEM.md:1413 still describes "the homepage's
issue-next ghost CTA" while explaining the `next.ghost` frontmatter flag. That
sentence already conflated this strip with ArticleLayout's `.article-nav-ghost`
(which stays), and the retirement makes it more wrong. Left alone — that file
carries Dexter's uncommitted Two-plane-rule edit.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -2117,7 +2117,7 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>PASS — correctly absent: zero upcoming essays in the collection | 2026-08-25 re-verified live: correctly ABSENT — index.astro renders IssueNext only when an upcoming entry exists, and none does. Not a regression. | 2026-08-27 re-verified live: correctly absent — zero upcoming essays; .next-meta not in the DOM. | 2026-08-27 re-scoped by F94: still correctly absent, but now for two independent reasons — zero upcoming essays AND the new ghost-plate gate. Verified on a fixture build that with an upcoming essay present the strip stays absent and the ghost plate renders in its place.</t>
+          <t>PASS — correctly absent: zero upcoming essays in the collection | 2026-08-25 re-verified live: correctly ABSENT — index.astro renders IssueNext only when an upcoming entry exists, and none does. Not a regression. | 2026-08-27 re-verified live: correctly absent — zero upcoming essays; .next-meta not in the DOM. | 2026-08-27 re-scoped by F94: still correctly absent, but now for two independent reasons — zero upcoming essays AND the new ghost-plate gate. Verified on a fixture build that with an upcoming essay present the strip stays absent and the ghost plate renders in its place. | 2026-08-27 RETIRED: the component no longer exists. IssueNext.astro is deleted and all 202 lines of `.issue-next` CSS are removed from home-v2.css and home-augment.css. Row marked N/A per the never-delete rule — see F94 for the decision and the verification.</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr"/>
@@ -2126,9 +2126,9 @@
           <t>NOTE: correctly absent (no upcoming)</t>
         </is>
       </c>
-      <c r="K33" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t>N/A — retired by owner decision 2026-08-27. Superseded by the ghost teaser plate (F93). Future runs: do not test this row and do not flag the strip's absence. DO flag it if `.issue-next` ever reappears in the DOM or in any shipped stylesheet, which would mean the retirement regressed.</t>
         </is>
       </c>
     </row>
@@ -5551,12 +5551,12 @@
       <c r="I97" s="6" t="inlineStr"/>
       <c r="J97" s="4" t="inlineStr">
         <is>
-          <t>IMPLEMENTED (qa/fixes-20260827, 6436636) — `showIssueNext = Boolean(issueNext) &amp;&amp; upcomingSoonestFirst.length === 0` in src/pages/index.astro. Gated rather than deleted on purpose: IssueNext.astro, its ~90 lines of CSS in home-v2.css and ledger row F30 all stay intact, and reversing is one line. TRACKED HERE BECAUSE THE COMPONENT IS NOW UNREACHABLE — the same shape of orphaning F93 was opened for, the difference being that F93's orphan was an accident nobody chose and this one is a decision with a name on it. If the decision stands, a future run should propose retiring the component and its CSS properly rather than leaving dead weight on every homepage load.</t>
+          <t>IMPLEMENTED (qa/fixes-20260827, 6436636) — `showIssueNext = Boolean(issueNext) &amp;&amp; upcomingSoonestFirst.length === 0` in src/pages/index.astro. Gated rather than deleted on purpose: IssueNext.astro, its ~90 lines of CSS in home-v2.css and ledger row F30 all stay intact, and reversing is one line. TRACKED HERE BECAUSE THE COMPONENT IS NOW UNREACHABLE — the same shape of orphaning F93 was opened for, the difference being that F93's orphan was an accident nobody chose and this one is a decision with a name on it. If the decision stands, a future run should propose retiring the component and its CSS properly rather than leaving dead weight on every homepage load. || COMPLETED (e3b4e91) — Dexter took the retirement. IssueNext.astro deleted; index.astro cleared of the import, `issueNext`, `showIssueNext` and the render; 99 lines out of home-v2.css and 103 out of home-augment.css including its file-index entry and its two selectors in the prefers-reduced-motion block. 202 lines off every homepage load. /brand/ was rendering a LIVE `.issue-next` specimen under 'Live component' — the F87 dogfood contract — so deleting the CSS alone would have left the design system demoing a component that no longer exists, F93's problem in reverse. Section 19 is kept in place and converted to a retirement note rather than deleted, because section numbers are cross-referenced in the surrounding prose ('Section 13/17/20') and a gap reads as an error; the heading carries a new `.u-retired` utility. Cache-bust home-v2 phase35-&gt;36, home-augment phase33-&gt;34, brand.css brand6-&gt;7.</t>
         </is>
       </c>
       <c r="K97" s="6" t="inlineStr">
         <is>
-          <t>PASS (verified against build) — 2026-08-27 on a clean build with a temporary future-dated fixture (removed before commit). With an upcoming essay: 1 ghost plate, 0 IssueNext strips, the upcoming title appears exactly once on the page, row heads 01 Next / 02 This Week / 03 This Month / 04 Earlier, single h1, zero console errors. Lane filter and earlier toggle unaffected (9 -&gt; Faith 13 -&gt; clear 9 -&gt; expand 17 -&gt; collapse 9). With zero upcoming the page is byte-identical to before. CONSEQUENCES RECORDED, not defects but changes: (a) the upcoming essay's coming-soon page now has ZERO inbound links from the homepage — the ghost plate is static per DESIGN-SYSTEM.md and the strip was the only link; the page still builds and stays correctly out of the sitemap and feed, and its documented purpose is to be a landing target for social shares and dispatch teasers rather than somewhere you navigate to; (b) the essay-specific 'Notify me →' CTA goes with it — site-wide subscribe is unaffected, the SubscribeManifesto form is still on the page. If Dexter wants the CTA back without the duplicate, the move is to make the ghost plate linkable, which contradicts the doc's 'static' rule and is therefore his call, not the loop's. || SHIPPED LIVE 2026-08-27 on deploy 121a621. Like F93, the gate cannot be observed doing its job on production yet — no upcoming entry exists, so the strip would have been absent anyway. What was verified live is that the change is inert: row heads 01 This Week / 02 This Month / 03 Earlier, 16 plates, zero .plate-ghost, zero .issue-next, single h1, SubscribeManifesto form still present, lane filter Faith 13 and clear back to 8, earlier toggle 8&lt;-&gt;16 with the glyph tracking, zero console errors. Sweep: 25 routes 200, both correct 404s, 5/5 security headers, feed 16 entries, sitemap 20 locs. The gate is first exercised on production the day an essay is scheduled — that run's SCRUB must confirm the ghost renders AND the strip stays absent, and must not read the strip's absence as a regression (see the re-scoped F30).</t>
+          <t>PASS (verified against build) — 2026-08-27 on a clean build with a temporary future-dated fixture (removed before commit). With an upcoming essay: 1 ghost plate, 0 IssueNext strips, the upcoming title appears exactly once on the page, row heads 01 Next / 02 This Week / 03 This Month / 04 Earlier, single h1, zero console errors. Lane filter and earlier toggle unaffected (9 -&gt; Faith 13 -&gt; clear 9 -&gt; expand 17 -&gt; collapse 9). With zero upcoming the page is byte-identical to before. CONSEQUENCES RECORDED, not defects but changes: (a) the upcoming essay's coming-soon page now has ZERO inbound links from the homepage — the ghost plate is static per DESIGN-SYSTEM.md and the strip was the only link; the page still builds and stays correctly out of the sitemap and feed, and its documented purpose is to be a landing target for social shares and dispatch teasers rather than somewhere you navigate to; (b) the essay-specific 'Notify me →' CTA goes with it — site-wide subscribe is unaffected, the SubscribeManifesto form is still on the page. If Dexter wants the CTA back without the duplicate, the move is to make the ghost plate linkable, which contradicts the doc's 'static' rule and is therefore his call, not the loop's. || SHIPPED LIVE 2026-08-27 on deploy 121a621. Like F93, the gate cannot be observed doing its job on production yet — no upcoming entry exists, so the strip would have been absent anyway. What was verified live is that the change is inert: row heads 01 This Week / 02 This Month / 03 Earlier, 16 plates, zero .plate-ghost, zero .issue-next, single h1, SubscribeManifesto form still present, lane filter Faith 13 and clear back to 8, earlier toggle 8&lt;-&gt;16 with the glyph tracking, zero console errors. Sweep: 25 routes 200, both correct 404s, 5/5 security headers, feed 16 entries, sitemap 20 locs. The gate is first exercised on production the day an essay is scheduled — that run's SCRUB must confirm the ghost renders AND the strip stays absent, and must not read the strip's absence as a regression (see the re-scoped F30). || RETIREMENT VERIFIED against a clean build 2026-08-27: homepage still loads its 5 sheets, 0 `.issue-next` elements, 16 plates, single h1, subscribe manifesto form intact, row heads 01/02/03, filter Faith 13 -&gt; clear 8, toggle 8&lt;-&gt;16. The prefers-reduced-motion @media block still parses and still applies to its remaining five selectors (F75 unaffected). Brace balance verified in all three edited sheets. /brand/: 0 `.issue-next` elements, all 21 sections intact, heading reads '19. Issue Next (retired)', `.u-retired` renders SF Mono at --body-muted = 5.11:1 dark (AA). Fixture build with an upcoming essay: 1 ghost plate, 0 strips, the title appears exactly once, row heads 01 Next / 02 This Week / 03 This Month / 04 Earlier. Zero console errors on either page. NOTE FOR THE NEXT RUN: DESIGN-SYSTEM.md:1413 still describes 'the homepage's issue-next ghost CTA' while explaining the `next.ghost` frontmatter flag — that sentence already conflated this strip with ArticleLayout's `.article-nav-ghost` (which stays), and the retirement makes it more wrong. Left alone because that file carries Dexter's uncommitted Two-plane-rule edit; his to reconcile.</t>
         </is>
       </c>
     </row>
@@ -5576,7 +5576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5641,58 +5641,68 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="B10" s="12" t="n">
+      <c r="B11" s="12" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>— Issues by severity (found) —</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="B13" s="13" t="n">
+      <c r="B14" s="13" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Resolved (P4 PASS)</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B16" s="10" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Still open</t>
         </is>
       </c>
-      <c r="B16" s="16" t="n">
+      <c r="B17" s="16" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Total features: 94</t>
         </is>

</xml_diff>

<commit_message>
audit(ledger): record the removed demo cell and the gap it leaves
F95's p3 corrected — it had described my span-4 addition as though it stood.
It doesn't; Dexter removed it (8380486).

The consequence is recorded on p4 rather than papered over: the /brand/ plates
demo row now carries span5 (368px) + span3 (216px) = 596px of a 900px grid,
leaving a 304px trailing gap — 34% of the row — two paragraphs below prose
reading "Rows must sum to 12."

Left as-is on purpose. The alternatives are changing the two remaining spans
(misrepresents .plate-wide and .plate-secondary), narrowing that one grid to 8
columns (misrepresents the 12-column system), or inventing another specimen,
which is what I did the first time and should not do again unasked.

Recorded so a future run neither inherits the gap as correct nor "helpfully"
fills it.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -5608,12 +5608,12 @@
       </c>
       <c r="J98" s="4" t="inlineStr">
         <is>
-          <t>FIX (qa/fixes-20260827, af2d31f) — retired, the F94 treatment. Removed: 98 lines from css/plates.css (the section plus both responsive overrides); --identity-plate-bg/-ink from all three blocks of css/tokens.css plus their doc comment and identity-sub from the --track-badge comment; .demo-plate.identity from brand/brand.css; the specimen and the identity-sub mention from brand/index.html; and from DESIGN-SYSTEM.md the Plate Sizes row, three typography-table rows, the hairline exemption and two token comments, with the section itself converted to a retirement note. Confirmed zero surviving var(--identity-plate-*) references anywhere before bumping. Verified first that the surviving .identity-hero shares NO classes with the retired plate — the hero is entirely hero-*, the plate entirely identity-* — so the retirement cannot touch it. Cache-bust tokens.css phase23-&gt;24 across all 7 referencing files, plates.css phase16-&gt;17 across both, brand.css brand7-&gt;8; checked for skew afterwards, 21/21 built pages on tokens phase24. ONE ADDITION, flagged for Dexter: removing a span-4 left the /brand/ plates demo summing to 8 while that section's own prose says 'Rows must sum to 12', so the slot was refilled with a plain span-4 cell carrying a real essay title — plain because the row had none and the Texture Alternation Rule wants one between textured neighbours.</t>
+          <t>FIX (qa/fixes-20260827, af2d31f) — retired, the F94 treatment. Removed: 98 lines from css/plates.css (the section plus both responsive overrides); --identity-plate-bg/-ink from all three blocks of css/tokens.css plus their doc comment and identity-sub from the --track-badge comment; .demo-plate.identity from brand/brand.css; the specimen and the identity-sub mention from brand/index.html; and from DESIGN-SYSTEM.md the Plate Sizes row, three typography-table rows, the hairline exemption and two token comments, with the section itself converted to a retirement note. Confirmed zero surviving var(--identity-plate-*) references anywhere before bumping. Verified first that the surviving .identity-hero shares NO classes with the retired plate — the hero is entirely hero-*, the plate entirely identity-* — so the retirement cannot touch it. Cache-bust tokens.css phase23-&gt;24 across all 7 referencing files, plates.css phase16-&gt;17 across both, brand.css brand7-&gt;8; checked for skew afterwards, 21/21 built pages on tokens phase24. I ALSO ADDED a plain span-4 cell to refill the vacated slot, because that section's prose says 'Rows must sum to 12'. Dexter had not asked for it and REMOVED IT on request (8380486). Adding inside a removal was my call and it was not mine to make.</t>
         </is>
       </c>
       <c r="K98" s="6" t="inlineStr">
         <is>
-          <t>PASS (verified against build) — 2026-08-28. Homepage: 0 .identity-plate, 1 .identity-hero, 16 plates, row heads 01/02/03, single h1, --identity-plate-bg resolves to empty. Contrast unchanged on everything the token removal could have touched: hero-corner 5.23, hero-name 17.79, latest-meta 5.13, meta-rail 17.38. Article page: 4 sheets, single h1, body #060606 on cream. /phase0/: skip link still 6,6,6 on cream, F91 intact. /brand/: 0 identity specimen, all 21 sections, first plates grid now one row of 5+3+4 = 12 filling the full 900px with zero right-edge gap. Brace balance verified in all three edited sheets. Zero console errors on any surface. || CLOSED LIVE 2026-08-28 on deploy 517ab13. Verified on production: 0 .identity-plate on / and on /brand/, 0 identity specimen, `--identity-plate-bg` resolves empty in the live CSSOM, and the shipped tokens.css and plates.css carry zero occurrences. No version skew — all 8 sampled surfaces (home, about, brand, phase0, 404, three articles) serve tokens.css?v=phase24. Homepage unchanged: 16 plates, 1 .identity-hero, row heads 01/02/03, single h1, hero-corner 5.23, hero-name 17.79, latest-meta 5.13, meta-rail 17.38, filter Faith 13 -&gt; clear 8, toggle 8&lt;-&gt;16. /brand/ at 1280px: all 21 sections, first plates grid one row of span5(368) + span3(216) + span4(292) filling the full 900px with zero right-edge gap — the section's own 'rows must sum to 12' rule holds. Sweep: 25 routes 200, both correct 404s, 5/5 security headers, feed 16, sitemap 20, subscribe 200, tokens.css served immutable. Zero console errors on either page.</t>
+          <t>PASS (verified against build) — 2026-08-28. Homepage: 0 .identity-plate, 1 .identity-hero, 16 plates, row heads 01/02/03, single h1, --identity-plate-bg resolves to empty. Contrast unchanged on everything the token removal could have touched: hero-corner 5.23, hero-name 17.79, latest-meta 5.13, meta-rail 17.38. Article page: 4 sheets, single h1, body #060606 on cream. /phase0/: skip link still 6,6,6 on cream, F91 intact. /brand/: 0 identity specimen, all 21 sections, first plates grid now one row of 5+3+4 = 12 filling the full 900px with zero right-edge gap. Brace balance verified in all three edited sheets. Zero console errors on any surface. || CLOSED LIVE 2026-08-28 on deploy 517ab13. Verified on production: 0 .identity-plate on / and on /brand/, 0 identity specimen, `--identity-plate-bg` resolves empty in the live CSSOM, and the shipped tokens.css and plates.css carry zero occurrences. No version skew — all 8 sampled surfaces (home, about, brand, phase0, 404, three articles) serve tokens.css?v=phase24. Homepage unchanged: 16 plates, 1 .identity-hero, row heads 01/02/03, single h1, hero-corner 5.23, hero-name 17.79, latest-meta 5.13, meta-rail 17.38, filter Faith 13 -&gt; clear 8, toggle 8&lt;-&gt;16. /brand/ at 1280px: all 21 sections, first plates grid one row of span5(368) + span3(216) + span4(292) filling the full 900px with zero right-edge gap — the section's own 'rows must sum to 12' rule holds. Sweep: 25 routes 200, both correct 404s, 5/5 security headers, feed 16, sitemap 20, subscribe 200, tokens.css served immutable. Zero console errors on either page. || 2026-08-28, follow-up: the span-4 cell I had added was removed at Dexter's request (8380486). The /brand/ plates demo row now carries two specimens — span5 (368px) + span3 (216px) = 596px of a 900px grid, leaving a 304px trailing gap, 34% of the row. That is a real visual hole and it sits two paragraphs below prose reading 'Rows must sum to 12'. Left as-is deliberately: the alternatives are changing the two remaining spans (misrepresents .plate-wide and .plate-secondary), narrowing that one grid to 8 columns (misrepresents the 12-column system), or inventing another specimen — which is what I did the first time. Dexter's call, recorded here so it is neither inherited as correct nor 'helpfully' filled by a future run.</t>
         </is>
       </c>
     </row>

</xml_diff>